<commit_message>
Modify UAT Test commition
</commit_message>
<xml_diff>
--- a/docs/UAT-commission-plans.xlsx
+++ b/docs/UAT-commission-plans.xlsx
@@ -16,6 +16,7 @@
     <sheet name="5 Generation" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="6 Affiliate" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="7 ล็อกแผน" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="8 จ่ายเงิน" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="215">
   <si>
     <t xml:space="preserve">UAT — ตรวจการตั้งค่าและการแบ่งค่าคอมทั้ง 6 แผน</t>
   </si>
@@ -78,10 +79,16 @@
     <t xml:space="preserve">ราคาสินค้า ฿10,000.00 · PV ฿7,000.00 · อัตราผู้ขาย 10% · หัวหน้า 5/3/1% — เลือกให้คิดเลขในใจได้ ไม่ใช่ข้อเสนอว่าบริษัทจริงควรจ่ายเท่าไร (BR-7)</t>
   </si>
   <si>
+    <t xml:space="preserve">ตั้งจ่ายเงินได้เลย</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตัวแทน UAT ทุกคนถูกกรอกบัญชีธนาคารและเอกสารยืนยันตัวตนไว้ให้แล้ว จึงขึ้นในคิว 'ตั้งจ่ายได้เลย' ได้ทันที — เลขบัญชีและเลขเอกสารขึ้นต้นด้วย UAT ทั้งหมด และเป็นหนังสือเดินทางไม่ใช่เลขบัตรประชาชน จึงไม่มีทางชนกับข้อมูลของคนจริง (ดูชีต 8)</t>
+  </si>
+  <si>
     <t xml:space="preserve">ยังไม่ครอบคลุม</t>
   </si>
   <si>
-    <t xml:space="preserve">ภาษีหัก ณ ที่จ่าย · การถอนเงิน · การคืนเงินและการกลับรายการ · ค่าคอมต่ออายุ · การแบ่งค่าคอมกับผู้ขายร่วม — แต่ละเรื่องมีทางเดินของตัวเองและควรมีชุดทดสอบแยก</t>
+    <t xml:space="preserve">การคืนเงินและการกลับรายการ · ค่าคอมต่ออายุ · การแบ่งค่าคอมกับผู้ขายร่วม — แต่ละเรื่องมีทางเดินของตัวเองและควรมีชุดทดสอบแยก</t>
   </si>
   <si>
     <t xml:space="preserve">สรุปผลรวมทุกแผน</t>
@@ -504,6 +511,12 @@
     <t xml:space="preserve">โหมด</t>
   </si>
   <si>
+    <t xml:space="preserve">ภาษีหัก ณ ที่จ่าย</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.00%  ← บริษัทเดียวที่หัก ที่อื่นไม่หัก</t>
+  </si>
+  <si>
     <t xml:space="preserve">ผู้ขาย → ผู้แนะนำ</t>
   </si>
   <si>
@@ -522,6 +535,9 @@
     <t xml:space="preserve">· ลองสลับเป็นโหมด deductive: ผู้ขายต้องเหลือ ฿700 และยอดจ่ายออกรวมต้องเท่าเดิมที่ ฿1,000</t>
   </si>
   <si>
+    <t xml:space="preserve">· บริษัทนี้หักภาษี ณ ที่จ่าย 3% — ยอดในตารางนี้คือยอดก่อนหัก ดูยอดโอนจริงในชีต 8</t>
+  </si>
+  <si>
     <t xml:space="preserve">ล็อกแผนเมื่อบริษัทขายไปแล้ว</t>
   </si>
   <si>
@@ -595,6 +611,69 @@
   </si>
   <si>
     <t xml:space="preserve">· ช่องสีเหลืองคือช่องที่ผู้ทดสอบกรอก ช่องอื่นเป็นค่าที่คาดไว้ อย่าแก้</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตั้งจ่าย → ตรวจสอบ → โอน</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ตัวแทน UAT ทุกคนมีบัญชีธนาคารและเอกสารยืนยันตัวตนครบแล้ว จึงขึ้นในคิว 'ตั้งจ่ายได้เลย' ได้ · เลขบัญชีและเลขเอกสารขึ้นต้นด้วย UAT และเป็นหนังสือเดินทางไม่ใช่เลขบัตรประชาชน จึงไม่มีทางชนกับข้อมูลของคนจริงในระบบค้นหา</t>
+  </si>
+  <si>
+    <t xml:space="preserve">แถบเหลือง 'มีค่าแนะนำ แต่ตั้งจ่ายไม่ได้' ต้องหายไป และทั้ง 4 คนย้ายมาอยู่ขั้นที่ 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UAT · Unilevel → จ่ายค่าแนะนำ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ขั้นที่ 1 ต้องขึ้น 4 คน รวม ฿1,900</t>
+  </si>
+  <si>
+    <t xml:space="preserve">หน้าเดียวกัน</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ติ๊กทั้ง 4 คนแล้วตั้งจ่าย → ต้องย้ายไปขั้นที่ 2 'รอคุณตรวจสอบ' ครบ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">อนุมัติ → ย้ายไปขั้นที่ 3 'รอฝ่ายบัญชีโอน' · ยอดยังเท่าเดิม</t>
+  </si>
+  <si>
+    <t xml:space="preserve">บันทึกการโอน → ย้ายไป 'โอนแล้ว' และแถวในบัญชีเปลี่ยนเป็นจ่ายแล้ว</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ขั้นที่ 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ไฟล์ CSV สำหรับโอน ดาวน์โหลดได้และมีเลขบัญชี UAT ครบทุกคน</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ปุ่มมุมขวาบน</t>
+  </si>
+  <si>
+    <t xml:space="preserve">บริษัท Affiliate หักภาษี ณ ที่จ่าย 3% — ยอดที่ได้ ฿1,000 ต้องโอนจริง ฿970 และหน้าจอต้องบอกทั้งสองยอด</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UAT · Affiliate → จ่ายค่าแนะนำ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">อีกห้าบริษัทต้องไม่มีบรรทัดภาษีเลย (ไม่ใช่ขึ้น 0.00)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">บริษัทอื่น ๆ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ลองลบบัญชีธนาคารของตัวแทนหนึ่งคนออก → เขาต้องหลุดจากขั้นที่ 1 กลับไปอยู่แถบเหลืองทันที</t>
+  </si>
+  <si>
+    <t xml:space="preserve">จัดการผู้ใช้ระบบ → กลับมาหน้าจ่าย</t>
+  </si>
+  <si>
+    <t xml:space="preserve">· อัตราภาษี 3% เป็นค่าทดสอบ ไม่ใช่ข้อเสนอว่าควรหักเท่าไร (BR-7) — อัตราจริงยังรอคุณกำหนด</t>
+  </si>
+  <si>
+    <t xml:space="preserve">· ข้อ 9 เป็นการทดสอบย้อนทาง: ด่านกันโอนเงินต้องปิดกลับได้ ไม่ใช่เปิดแล้วเปิดค้าง</t>
+  </si>
+  <si>
+    <t xml:space="preserve">· การคืนเงินและการกลับรายการค่าคอมยังไม่อยู่ในชุดนี้ — เป็นทางเดินอีกเส้นและควรมีชุดทดสอบแยก</t>
   </si>
 </sst>
 </file>
@@ -1114,7 +1193,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:C31"/>
+  <dimension ref="A2:C33"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
@@ -1188,7 +1267,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B19" s="3" t="s">
         <v>16</v>
       </c>
@@ -1196,36 +1275,26 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="5" t="s">
+    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B21" s="3" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6"/>
-      <c r="B23" s="6" t="s">
+      <c r="C21" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="6" t="s">
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="7" t="s">
+    <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6"/>
+      <c r="B25" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C24" s="8" t="n">
-        <f aca="false">SUM('1 Unilevel'!D18:D21)</f>
-        <v>1900</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="7" t="s">
+      <c r="C25" s="6" t="s">
         <v>22</v>
-      </c>
-      <c r="C25" s="8" t="n">
-        <f aca="false">SUM('2 Binary'!D18:D20)</f>
-        <v>3000</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1233,8 +1302,8 @@
         <v>23</v>
       </c>
       <c r="C26" s="8" t="n">
-        <f aca="false">SUM('3 Matrix'!D18:D20)</f>
-        <v>1260</v>
+        <f aca="false">SUM('1 Unilevel'!D18:D21)</f>
+        <v>1900</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1242,8 +1311,8 @@
         <v>24</v>
       </c>
       <c r="C27" s="8" t="n">
-        <f aca="false">SUM('4 Stairstep'!D17:D19)</f>
-        <v>1500</v>
+        <f aca="false">SUM('2 Binary'!D18:D20)</f>
+        <v>3000</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1251,8 +1320,8 @@
         <v>25</v>
       </c>
       <c r="C28" s="8" t="n">
-        <f aca="false">SUM('5 Generation'!D17:D21)</f>
-        <v>1800</v>
+        <f aca="false">SUM('3 Matrix'!D18:D20)</f>
+        <v>1260</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1260,13 +1329,31 @@
         <v>26</v>
       </c>
       <c r="C29" s="8" t="n">
-        <f aca="false">SUM('6 Affiliate'!D16:D17)</f>
+        <f aca="false">SUM('4 Stairstep'!D17:D19)</f>
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="C30" s="8" t="n">
+        <f aca="false">SUM('5 Generation'!D17:D21)</f>
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="C31" s="8" t="n">
+        <f aca="false">SUM('6 Affiliate'!D17:D18)</f>
         <v>1300</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C31" s="2" t="s">
-        <v>27</v>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C33" s="2" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1298,33 +1385,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
@@ -1332,176 +1419,176 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C14" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D18" s="12" t="n">
         <v>1000</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D19" s="12" t="n">
         <v>500</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B20" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="B20" s="11" t="s">
-        <v>61</v>
-      </c>
       <c r="C20" s="11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D20" s="12" t="n">
         <v>300</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D21" s="12" t="n">
         <v>100</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C22" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D22" s="14" t="n">
         <f aca="false">SUM(D18:D21)</f>
@@ -1510,12 +1597,12 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
@@ -1525,7 +1612,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B26" s="15"/>
       <c r="C26" s="15"/>
@@ -1535,7 +1622,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1604,33 +1691,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
@@ -1638,158 +1725,158 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C14" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D18" s="12" t="n">
         <v>1000</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D19" s="12" t="n">
         <v>1000</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D20" s="12" t="n">
         <v>1000</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C21" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D21" s="14" t="n">
         <f aca="false">SUM(D18:D20)</f>
@@ -1798,12 +1885,12 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
@@ -1813,7 +1900,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
@@ -1823,7 +1910,7 @@
     </row>
     <row r="26" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B26" s="15"/>
       <c r="C26" s="15"/>
@@ -1833,7 +1920,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B27" s="15"/>
       <c r="C27" s="15"/>
@@ -1843,7 +1930,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1914,33 +2001,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
@@ -1948,158 +2035,158 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C14" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D18" s="12" t="n">
         <v>700</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D19" s="12" t="n">
         <v>350</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="B20" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="B20" s="11" t="s">
-        <v>106</v>
-      </c>
       <c r="C20" s="11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D20" s="12" t="n">
         <v>210</v>
       </c>
       <c r="E20" s="11" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C21" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D21" s="14" t="n">
         <f aca="false">SUM(D18:D20)</f>
@@ -2108,12 +2195,12 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
@@ -2123,7 +2210,7 @@
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
@@ -2133,7 +2220,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B26" s="15"/>
       <c r="C26" s="15"/>
@@ -2143,7 +2230,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2213,33 +2300,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
@@ -2247,149 +2334,149 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C13" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D17" s="12" t="n">
         <v>500</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D18" s="12" t="n">
         <v>500</v>
       </c>
       <c r="E18" s="11" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
+        <v>130</v>
+      </c>
+      <c r="B19" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="B19" s="11" t="s">
-        <v>126</v>
-      </c>
       <c r="C19" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D19" s="12" t="n">
         <v>500</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C20" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D20" s="14" t="n">
         <f aca="false">SUM(D17:D19)</f>
@@ -2398,12 +2485,12 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B23" s="15"/>
       <c r="C23" s="15"/>
@@ -2413,7 +2500,7 @@
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
@@ -2423,7 +2510,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
@@ -2433,7 +2520,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2503,33 +2590,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
@@ -2537,185 +2624,185 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C13" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D17" s="12" t="n">
         <v>1000</v>
       </c>
       <c r="E17" s="11" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F17" s="10"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D18" s="18" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D19" s="12" t="n">
         <v>500</v>
       </c>
       <c r="E19" s="11" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F19" s="10"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D20" s="18" t="n">
         <v>0</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D21" s="12" t="n">
         <v>300</v>
       </c>
       <c r="E21" s="11" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="F21" s="10"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C22" s="13" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D22" s="14" t="n">
         <f aca="false">SUM(D17:D21)</f>
@@ -2724,12 +2811,12 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="15" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B25" s="15"/>
       <c r="C25" s="15"/>
@@ -2739,7 +2826,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="15" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B26" s="15"/>
       <c r="C26" s="15"/>
@@ -2749,7 +2836,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="15" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B27" s="15"/>
       <c r="C27" s="15"/>
@@ -2759,7 +2846,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2816,7 +2903,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -2829,33 +2916,33 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
@@ -2863,146 +2950,145 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C11" s="10"/>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>48</v>
+        <v>160</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="C12" s="10"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B15" s="6" t="s">
+      <c r="B13" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="C13" s="10"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C15" s="6" t="s">
+    </row>
+    <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="B16" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="C16" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="D16" s="6" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="s">
+      <c r="E16" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="F16" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C16" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="D16" s="12" t="n">
-        <v>1000</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="F16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>160</v>
+        <v>59</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D17" s="12" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="F17" s="10"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="D18" s="12" t="n">
         <v>300</v>
       </c>
-      <c r="E17" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="F17" s="10"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="D18" s="14" t="n">
-        <f aca="false">SUM(D16:D17)</f>
+      <c r="E18" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="F18" s="10"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C19" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="D19" s="14" t="n">
+        <f aca="false">SUM(D17:D18)</f>
         <v>1300</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B22" s="15"/>
       <c r="C22" s="15"/>
@@ -3010,26 +3096,30 @@
       <c r="E22" s="15"/>
       <c r="F22" s="15"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="16"/>
-      <c r="B25" s="16"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="B23" s="15"/>
+      <c r="C23" s="15"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="15"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15"/>
+      <c r="D24" s="15"/>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="16"/>
-      <c r="B26" s="16"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
+      <c r="A26" s="5" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="16"/>
@@ -3047,11 +3137,28 @@
       <c r="E28" s="16"/>
       <c r="F28" s="16"/>
     </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="16"/>
+      <c r="B29" s="16"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="16"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="16"/>
+      <c r="B30" s="16"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="16"/>
+      <c r="E30" s="16"/>
+      <c r="F30" s="16"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A21:F21"/>
+  <mergeCells count="4">
     <mergeCell ref="A22:F22"/>
-    <mergeCell ref="A25:F28"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A27:F30"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -3079,26 +3186,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3106,10 +3213,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D5" s="10"/>
     </row>
@@ -3118,10 +3225,10 @@
         <v>2</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="D6" s="10"/>
     </row>
@@ -3130,10 +3237,10 @@
         <v>3</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="D7" s="10"/>
     </row>
@@ -3142,10 +3249,10 @@
         <v>4</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="D8" s="10"/>
     </row>
@@ -3154,10 +3261,10 @@
         <v>5</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="D9" s="10"/>
     </row>
@@ -3166,10 +3273,10 @@
         <v>6</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="D10" s="10"/>
     </row>
@@ -3178,10 +3285,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="D11" s="10"/>
     </row>
@@ -3190,10 +3297,10 @@
         <v>8</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="D12" s="10"/>
     </row>
@@ -3202,21 +3309,21 @@
         <v>9</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="D13" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="19" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="B17" s="19"/>
       <c r="C17" s="19"/>
@@ -3224,7 +3331,7 @@
     </row>
     <row r="18" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="19" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="B18" s="19"/>
       <c r="C18" s="19"/>
@@ -3243,4 +3350,195 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="62"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="D5" s="10"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="D6" s="10"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="D7" s="10"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>201</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>177</v>
+      </c>
+      <c r="D8" s="10"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="D9" s="10"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>204</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="D10" s="10"/>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="D11" s="10"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>209</v>
+      </c>
+      <c r="D12" s="10"/>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="D13" s="10"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="19" t="s">
+        <v>212</v>
+      </c>
+      <c r="B17" s="19"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+    </row>
+    <row r="18" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="19" t="s">
+        <v>213</v>
+      </c>
+      <c r="B18" s="19"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="19"/>
+    </row>
+    <row r="19" customFormat="false" ht="12.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="19" t="s">
+        <v>214</v>
+      </c>
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A18:D18"/>
+    <mergeCell ref="A19:D19"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>